<commit_message>
Add new fields to PIN-level data in IC reference files
</commit_message>
<xml_diff>
--- a/dbt/export/templates/qc.vw_ic_reference_all_non_res_pin_level_data.xlsx
+++ b/dbt/export/templates/qc.vw_ic_reference_all_non_res_pin_level_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jecochr\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9551BCBE-A01A-4853-A465-1AFFBF3C8EC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6EC2074-F94A-4B47-B476-32F935B0E725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1860" yWindow="3732" windowWidth="23040" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Query Results" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="35">
   <si>
     <t>PARDAT</t>
   </si>
@@ -119,6 +119,12 @@
   </si>
   <si>
     <t>VALASM3</t>
+  </si>
+  <si>
+    <t>ECF</t>
+  </si>
+  <si>
+    <t>Exemption</t>
   </si>
 </sst>
 </file>
@@ -491,10 +497,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AD2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AF2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -529,10 +535,10 @@
         <v>1</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>2</v>
@@ -550,10 +556,10 @@
         <v>2</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>0</v>
@@ -562,10 +568,10 @@
         <v>0</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Y1" s="1" t="s">
         <v>3</v>
@@ -577,16 +583,22 @@
         <v>3</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="AD1" s="1" t="s">
         <v>26</v>
       </c>
+      <c r="AE1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -621,60 +633,66 @@
         <v>14</v>
       </c>
       <c r="L2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="N2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="Q2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="R2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="1" t="s">
+      <c r="S2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="R2" s="1" t="s">
+      <c r="T2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="U2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="T2" s="1" t="s">
+      <c r="V2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="U2" s="1" t="s">
+      <c r="W2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="V2" s="1" t="s">
+      <c r="X2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="W2" s="1" t="s">
+      <c r="Y2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="X2" s="1" t="s">
+      <c r="Z2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="Y2" s="1" t="s">
+      <c r="AA2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="Z2" s="1" t="s">
+      <c r="AB2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AA2" s="1" t="s">
+      <c r="AC2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="AB2" s="1" t="s">
+      <c r="AD2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AC2" s="1" t="s">
+      <c r="AE2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AD2" s="1" t="s">
+      <c r="AF2" s="1" t="s">
         <v>32</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add new fields to PIN-level data in IC reference files (#1067)
</commit_message>
<xml_diff>
--- a/dbt/export/templates/qc.vw_ic_reference_all_non_res_pin_level_data.xlsx
+++ b/dbt/export/templates/qc.vw_ic_reference_all_non_res_pin_level_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jecochr\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9551BCBE-A01A-4853-A465-1AFFBF3C8EC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6EC2074-F94A-4B47-B476-32F935B0E725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1860" yWindow="3732" windowWidth="23040" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Query Results" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="35">
   <si>
     <t>PARDAT</t>
   </si>
@@ -119,6 +119,12 @@
   </si>
   <si>
     <t>VALASM3</t>
+  </si>
+  <si>
+    <t>ECF</t>
+  </si>
+  <si>
+    <t>Exemption</t>
   </si>
 </sst>
 </file>
@@ -491,10 +497,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AD2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AF2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -529,10 +535,10 @@
         <v>1</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>2</v>
@@ -550,10 +556,10 @@
         <v>2</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>0</v>
@@ -562,10 +568,10 @@
         <v>0</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Y1" s="1" t="s">
         <v>3</v>
@@ -577,16 +583,22 @@
         <v>3</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="AD1" s="1" t="s">
         <v>26</v>
       </c>
+      <c r="AE1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -621,60 +633,66 @@
         <v>14</v>
       </c>
       <c r="L2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="N2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="Q2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="R2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="1" t="s">
+      <c r="S2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="R2" s="1" t="s">
+      <c r="T2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="U2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="T2" s="1" t="s">
+      <c r="V2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="U2" s="1" t="s">
+      <c r="W2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="V2" s="1" t="s">
+      <c r="X2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="W2" s="1" t="s">
+      <c r="Y2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="X2" s="1" t="s">
+      <c r="Z2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="Y2" s="1" t="s">
+      <c r="AA2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="Z2" s="1" t="s">
+      <c r="AB2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AA2" s="1" t="s">
+      <c r="AC2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="AB2" s="1" t="s">
+      <c r="AD2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AC2" s="1" t="s">
+      <c r="AE2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AD2" s="1" t="s">
+      <c r="AF2" s="1" t="s">
         <v>32</v>
       </c>
     </row>

</xml_diff>